<commit_message>
Fix time dilation inversion (gamma*m0 -> m0/gamma) in 4 cells: C92, G45, Q13, S13
Phase clock was multiplying by gamma instead of dividing, causing
unphysical frequency spike at relativistic speeds. Same Einstein Stick
bug that was fixed in the Python engine.

Source of truth: Z:\teleparallel_sim_photons\TEGR_10x10_Matrix_WORKING.xlsx
</commit_message>
<xml_diff>
--- a/TEGR_10x10_Matrix_WORKING.xlsx
+++ b/TEGR_10x10_Matrix_WORKING.xlsx
@@ -1530,14 +1530,14 @@
         <v>0</v>
       </c>
       <c r="Q13" s="29">
-        <f>C14*C28^2/C29</f>
+        <f>C28^2/(C14*C29)</f>
         <v/>
       </c>
       <c r="R13" s="10" t="n">
         <v>0</v>
       </c>
       <c r="S13" s="29">
-        <f>C12*C28^2/C29</f>
+        <f>-C12*C28^2/(C14^2*C29)</f>
         <v/>
       </c>
       <c r="T13" s="1" t="n"/>
@@ -2720,7 +2720,7 @@
         </is>
       </c>
       <c r="G45" s="30">
-        <f>C14*C12*C28^2/C29</f>
+        <f>(C12/C14)*C28^2/C29</f>
         <v/>
       </c>
       <c r="H45" s="3" t="inlineStr">
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C92" s="34">
-        <f>MOD(C13+C75*C12*C28^2/C29*C30, 2*PI())</f>
+        <f>MOD(C13+(C12/C75)*C28^2/C29*C30, 2*PI())</f>
         <v/>
       </c>
       <c r="D92" s="3" t="inlineStr">
@@ -4105,7 +4105,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B38"/>
+  <dimension ref="A1:S92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4400,6 +4400,8 @@
         </is>
       </c>
     </row>
+    <row r="45"/>
+    <row r="92"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4412,7 +4414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:S92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4434,7 +4436,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -4491,7 +4492,6 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
@@ -4553,7 +4553,6 @@
         <v/>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
@@ -4609,6 +4608,8 @@
         </is>
       </c>
     </row>
+    <row r="45"/>
+    <row r="92"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>